<commit_message>
Template contoh lebih lengkap + upload terbuka untuk semua user aktif
Template produk/supplier diperkaya (10 produk lintas kategori, 5 supplier).
/template bisa diunduh semua user whitelist (tanpa gate owner). kios_import_upload
kini boleh dipakai semua user aktif (bukan owner-only) — import non-destruktif
(update/create by nama, kolom kosong tak menimpa).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/produk-template.xlsx
+++ b/templates/produk-template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>nama</t>
   </si>
@@ -70,6 +70,9 @@
     <t>botol</t>
   </si>
   <si>
+    <t>Tepung Terigu 1kg</t>
+  </si>
+  <si>
     <t>Indomie Goreng</t>
   </si>
   <si>
@@ -80,6 +83,45 @@
   </si>
   <si>
     <t>Grosir Baa</t>
+  </si>
+  <si>
+    <t>Teh Botol 350ml</t>
+  </si>
+  <si>
+    <t>minuman</t>
+  </si>
+  <si>
+    <t>Kopi Sachet</t>
+  </si>
+  <si>
+    <t>renceng</t>
+  </si>
+  <si>
+    <t>Rokok Surya 16</t>
+  </si>
+  <si>
+    <t>rokok</t>
+  </si>
+  <si>
+    <t>Agen Rokok Rote</t>
+  </si>
+  <si>
+    <t>Gas LPG 3kg</t>
+  </si>
+  <si>
+    <t>gas</t>
+  </si>
+  <si>
+    <t>tabung</t>
+  </si>
+  <si>
+    <t>Pangkalan Gas Baa</t>
+  </si>
+  <si>
+    <t>Sabun Mandi</t>
+  </si>
+  <si>
+    <t>kebutuhan</t>
   </si>
 </sst>
 </file>
@@ -518,28 +560,202 @@
         <v>18</v>
       </c>
       <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5">
+        <v>18</v>
+      </c>
+      <c r="E5">
+        <v>11000</v>
+      </c>
+      <c r="F5">
+        <v>13000</v>
+      </c>
+      <c r="G5">
+        <v>8</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="D5">
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6">
         <v>50</v>
       </c>
-      <c r="E5">
+      <c r="E6">
         <v>2800</v>
       </c>
-      <c r="F5">
+      <c r="F6">
         <v>3500</v>
       </c>
-      <c r="G5">
+      <c r="G6">
         <v>20</v>
       </c>
-      <c r="H5">
+      <c r="H6">
         <v>5</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7">
+        <v>36</v>
+      </c>
+      <c r="E7">
+        <v>3000</v>
+      </c>
+      <c r="F7">
+        <v>4000</v>
+      </c>
+      <c r="G7">
+        <v>12</v>
+      </c>
+      <c r="H7">
+        <v>4</v>
+      </c>
+      <c r="I7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8">
+        <v>30</v>
+      </c>
+      <c r="E8">
+        <v>9000</v>
+      </c>
+      <c r="F8">
+        <v>11000</v>
+      </c>
+      <c r="G8">
+        <v>10</v>
+      </c>
+      <c r="H8">
+        <v>3</v>
+      </c>
+      <c r="I8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9">
+        <v>40</v>
+      </c>
+      <c r="E9">
+        <v>27000</v>
+      </c>
+      <c r="F9">
+        <v>29000</v>
+      </c>
+      <c r="G9">
+        <v>15</v>
+      </c>
+      <c r="H9">
+        <v>5</v>
+      </c>
+      <c r="I9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10">
+        <v>10</v>
+      </c>
+      <c r="E10">
+        <v>18000</v>
+      </c>
+      <c r="F10">
+        <v>22000</v>
+      </c>
+      <c r="G10">
+        <v>5</v>
+      </c>
+      <c r="H10">
+        <v>2</v>
+      </c>
+      <c r="I10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
         <v>21</v>
+      </c>
+      <c r="D11">
+        <v>25</v>
+      </c>
+      <c r="E11">
+        <v>3500</v>
+      </c>
+      <c r="F11">
+        <v>5000</v>
+      </c>
+      <c r="G11">
+        <v>10</v>
+      </c>
+      <c r="H11">
+        <v>3</v>
+      </c>
+      <c r="I11" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tambah kolom barcode ke produk (template, import, CRUD, cari)
Produk punya field barcode; bisa dicari/jual via barcode (CariProduk cocokkan
barcode persis). Template produk (.xlsx/.csv) tambah kolom barcode + contoh.
Didukung di tambah_produk, edit_produk, import file, dan tampilan detail.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/produk-template.xlsx
+++ b/templates/produk-template.xlsx
@@ -14,11 +14,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>nama</t>
   </si>
   <si>
+    <t>barcode</t>
+  </si>
+  <si>
     <t>kategori</t>
   </si>
   <si>
@@ -46,6 +49,9 @@
     <t>Beras Medium 5kg</t>
   </si>
   <si>
+    <t>8991234500015</t>
+  </si>
+  <si>
     <t>sembako</t>
   </si>
   <si>
@@ -58,6 +64,9 @@
     <t>Gula Pasir 1kg</t>
   </si>
   <si>
+    <t>8991234500022</t>
+  </si>
+  <si>
     <t>bungkus</t>
   </si>
   <si>
@@ -67,15 +76,24 @@
     <t>Minyak Goreng 1L</t>
   </si>
   <si>
+    <t>8991234500039</t>
+  </si>
+  <si>
     <t>botol</t>
   </si>
   <si>
     <t>Tepung Terigu 1kg</t>
   </si>
   <si>
+    <t>8991234500046</t>
+  </si>
+  <si>
     <t>Indomie Goreng</t>
   </si>
   <si>
+    <t>089686010947</t>
+  </si>
+  <si>
     <t>mie</t>
   </si>
   <si>
@@ -88,18 +106,27 @@
     <t>Teh Botol 350ml</t>
   </si>
   <si>
+    <t>8992761111118</t>
+  </si>
+  <si>
     <t>minuman</t>
   </si>
   <si>
     <t>Kopi Sachet</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>renceng</t>
   </si>
   <si>
     <t>Rokok Surya 16</t>
   </si>
   <si>
+    <t>8997011710018</t>
+  </si>
+  <si>
     <t>rokok</t>
   </si>
   <si>
@@ -119,6 +146,9 @@
   </si>
   <si>
     <t>Sabun Mandi</t>
+  </si>
+  <si>
+    <t>8999999036007</t>
   </si>
   <si>
     <t>kebutuhan</t>
@@ -436,7 +466,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="9" min="1" width="18"/>
+    <col customWidth="true" max="10" min="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,295 +497,328 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+      <c r="F2">
+        <v>55000</v>
+      </c>
+      <c r="G2">
+        <v>62000</v>
+      </c>
+      <c r="H2">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2">
-        <v>20</v>
-      </c>
-      <c r="E2">
-        <v>55000</v>
-      </c>
-      <c r="F2">
-        <v>62000</v>
-      </c>
-      <c r="G2">
-        <v>10</v>
-      </c>
-      <c r="H2">
+      <c r="I2">
         <v>3</v>
       </c>
-      <c r="I2" t="s">
-        <v>12</v>
+      <c r="J2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3">
         <v>15</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>13500</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>15000</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>8</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>2</v>
       </c>
-      <c r="I3" t="s">
-        <v>15</v>
+      <c r="J3" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4">
+        <v>24</v>
+      </c>
+      <c r="F4">
+        <v>16000</v>
+      </c>
+      <c r="G4">
+        <v>18000</v>
+      </c>
+      <c r="H4">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4">
-        <v>24</v>
-      </c>
-      <c r="E4">
-        <v>16000</v>
-      </c>
-      <c r="F4">
-        <v>18000</v>
-      </c>
-      <c r="G4">
-        <v>10</v>
-      </c>
-      <c r="H4">
+      <c r="I4">
         <v>3</v>
       </c>
-      <c r="I4" t="s">
-        <v>12</v>
+      <c r="J4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5">
+      <c r="F5">
+        <v>11000</v>
+      </c>
+      <c r="G5">
+        <v>13000</v>
+      </c>
+      <c r="H5">
+        <v>8</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5" t="s">
         <v>18</v>
-      </c>
-      <c r="E5">
-        <v>11000</v>
-      </c>
-      <c r="F5">
-        <v>13000</v>
-      </c>
-      <c r="G5">
-        <v>8</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6">
+        <v>50</v>
+      </c>
+      <c r="F6">
+        <v>2800</v>
+      </c>
+      <c r="G6">
+        <v>3500</v>
+      </c>
+      <c r="H6">
         <v>20</v>
       </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6">
-        <v>50</v>
-      </c>
-      <c r="E6">
-        <v>2800</v>
-      </c>
-      <c r="F6">
-        <v>3500</v>
-      </c>
-      <c r="G6">
-        <v>20</v>
-      </c>
-      <c r="H6">
+      <c r="I6">
         <v>5</v>
       </c>
-      <c r="I6" t="s">
-        <v>22</v>
+      <c r="J6" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7">
         <v>36</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>3000</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>4000</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>12</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>4</v>
       </c>
-      <c r="I7" t="s">
-        <v>22</v>
+      <c r="J7" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8">
         <v>30</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>9000</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>11000</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>10</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>3</v>
       </c>
-      <c r="I8" t="s">
-        <v>22</v>
+      <c r="J8" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9">
+        <v>37</v>
+      </c>
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9">
         <v>40</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>27000</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>29000</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>15</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>5</v>
       </c>
-      <c r="I9" t="s">
-        <v>29</v>
+      <c r="J9" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10">
+        <v>40</v>
+      </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10">
         <v>10</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>18000</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>22000</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>5</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>2</v>
       </c>
-      <c r="I10" t="s">
-        <v>33</v>
+      <c r="J10" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11">
+        <v>45</v>
+      </c>
+      <c r="D11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11">
         <v>25</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>3500</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <v>5000</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>10</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>3</v>
       </c>
-      <c r="I11" t="s">
-        <v>22</v>
+      <c r="J11" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload gambar manual, QR dinamis WhatsApp, kolom gambar impor
- Gambar QRIS & produk bisa diunggah manual: dikompres client-side jadi
  data URL (tanpa storage eksternal), tetap bisa tempel URL.
- Di /toko, saat pembeli pilih QRIS muncul tombol chat kasir via
  WhatsApp untuk minta QR dinamis sesuai total.
- Template impor Excel/CSV dapat kolom "gambar"; mapping image_url
  ditambahkan di impor dashboard (TS) & bot (Go).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/produk-template.xlsx
+++ b/templates/produk-template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>nama</t>
   </si>
@@ -46,6 +46,9 @@
     <t>supplier</t>
   </si>
   <si>
+    <t>gambar</t>
+  </si>
+  <si>
     <t>Beras Medium 5kg</t>
   </si>
   <si>
@@ -61,6 +64,9 @@
     <t>UD Maju</t>
   </si>
   <si>
+    <t>https://contoh.com/gambar/beras.jpg</t>
+  </si>
+  <si>
     <t>Gula Pasir 1kg</t>
   </si>
   <si>
@@ -73,6 +79,9 @@
     <t>Distributor Kupang</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>Minyak Goreng 1L</t>
   </si>
   <si>
@@ -113,9 +122,6 @@
   </si>
   <si>
     <t>Kopi Sachet</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>renceng</t>
@@ -466,7 +472,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="10" min="1" width="18"/>
+    <col customWidth="true" max="11" min="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,19 +506,22 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2">
         <v>20</v>
@@ -530,21 +539,24 @@
         <v>3</v>
       </c>
       <c r="J2" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="K2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E3">
         <v>15</v>
@@ -562,21 +574,24 @@
         <v>2</v>
       </c>
       <c r="J3" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="K3" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E4">
         <v>24</v>
@@ -594,21 +609,24 @@
         <v>3</v>
       </c>
       <c r="J4" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="K4" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E5">
         <v>18</v>
@@ -626,21 +644,24 @@
         <v>2</v>
       </c>
       <c r="J5" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="K5" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E6">
         <v>50</v>
@@ -658,21 +679,24 @@
         <v>5</v>
       </c>
       <c r="J6" t="s">
-        <v>28</v>
+        <v>31</v>
+      </c>
+      <c r="K6" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E7">
         <v>36</v>
@@ -690,21 +714,24 @@
         <v>4</v>
       </c>
       <c r="J7" t="s">
-        <v>28</v>
+        <v>31</v>
+      </c>
+      <c r="K7" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E8">
         <v>30</v>
@@ -722,21 +749,24 @@
         <v>3</v>
       </c>
       <c r="J8" t="s">
-        <v>28</v>
+        <v>31</v>
+      </c>
+      <c r="K8" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E9">
         <v>40</v>
@@ -754,21 +784,24 @@
         <v>5</v>
       </c>
       <c r="J9" t="s">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="K9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E10">
         <v>10</v>
@@ -786,21 +819,24 @@
         <v>2</v>
       </c>
       <c r="J10" t="s">
-        <v>42</v>
+        <v>44</v>
+      </c>
+      <c r="K10" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E11">
         <v>25</v>
@@ -818,7 +854,10 @@
         <v>3</v>
       </c>
       <c r="J11" t="s">
-        <v>28</v>
+        <v>31</v>
+      </c>
+      <c r="K11" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
QRIS pesanan via WhatsApp kirim QR dinamis manual + contoh snack template
Di menu Pesanan, pesan WhatsApp ke pembeli kini hanya berisi struk +
info bahwa QR dinamis dikirim sebagai foto; kartu pesanan QRIS memberi
pengingat agar kasir screenshot QR dinamis & lampirkan bersama struk
(link QR statis dihapus dari alur ini). Tambah baris contoh kategori
snack di template impor Excel/CSV.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/produk-template.xlsx
+++ b/templates/produk-template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>nama</t>
   </si>
@@ -158,6 +158,15 @@
   </si>
   <si>
     <t>kebutuhan</t>
+  </si>
+  <si>
+    <t>Biskuit Kelapa</t>
+  </si>
+  <si>
+    <t>8990111222333</t>
+  </si>
+  <si>
+    <t>snack</t>
   </si>
 </sst>
 </file>
@@ -860,6 +869,41 @@
         <v>21</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12">
+        <v>40</v>
+      </c>
+      <c r="F12">
+        <v>3500</v>
+      </c>
+      <c r="G12">
+        <v>5000</v>
+      </c>
+      <c r="H12">
+        <v>15</v>
+      </c>
+      <c r="I12">
+        <v>5</v>
+      </c>
+      <c r="J12" t="s">
+        <v>31</v>
+      </c>
+      <c r="K12" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ui): template Excel lebih baik + dashboard lebih responsif
- Excel: header navy-blue, lebar kolom spesifik, dropdown validasi
  (kategori & satuan), format angka #,##0, zebra row, border, 30 baris
  extra pre-styled
- produk-form: grid-cols-3 → grid-cols-2 sm:grid-cols-3 (tidak mepet di HP)
- kasir-form: tambah md:grid-cols-2 untuk tablet (50-50 split)
- penjualan-view: mobile card list di bawah sm, tabel hanya di sm+
- suplier-table: mobile card list di bawah md, tabel hanya di md+

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/produk-template.xlsx
+++ b/templates/produk-template.xlsx
@@ -173,7 +173,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -183,18 +183,34 @@
     <font>
       <family val="2"/>
       <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <family val="2"/>
       <color/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B4F72"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6EAF8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -202,14 +218,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFC9CA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFC9CA"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFC9CA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFC9CA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="false">
-      <alignment/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -481,10 +523,18 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="11" min="1" width="18"/>
+    <col customWidth="true" max="1" min="1" width="28"/>
+    <col customWidth="true" max="2" min="2" width="18"/>
+    <col customWidth="true" max="3" min="3" width="15"/>
+    <col customWidth="true" max="4" min="4" width="11"/>
+    <col customWidth="true" max="5" min="5" width="10"/>
+    <col customWidth="true" max="7" min="6" width="16"/>
+    <col customWidth="true" max="9" min="8" width="14"/>
+    <col customWidth="true" max="10" min="10" width="22"/>
+    <col customWidth="true" max="11" min="11" width="42"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="true">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -520,390 +570,788 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="3">
         <v>20</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="3">
         <v>55000</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="3">
         <v>62000</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="3">
         <v>10</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="3">
         <v>3</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
+      <c r="A3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="5">
         <v>15</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="5">
         <v>13500</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="5">
         <v>15000</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="5">
         <v>8</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="5">
         <v>2</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="3">
         <v>24</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="3">
         <v>16000</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="3">
         <v>18000</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="3">
         <v>10</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="3">
         <v>3</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s">
+      <c r="A5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="5">
         <v>18</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="5">
         <v>11000</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="5">
         <v>13000</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="5">
         <v>8</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="5">
         <v>2</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="3">
         <v>50</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="3">
         <v>2800</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="3">
         <v>3500</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="3">
         <v>20</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="3">
         <v>5</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s">
+      <c r="A7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="5">
         <v>36</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="5">
         <v>3000</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="5">
         <v>4000</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="5">
         <v>12</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="5">
         <v>4</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="3">
         <v>30</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="3">
         <v>9000</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="3">
         <v>11000</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="3">
         <v>10</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="3">
         <v>3</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="s">
+      <c r="A9" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="5">
         <v>40</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="5">
         <v>27000</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="5">
         <v>29000</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="5">
         <v>15</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="5">
         <v>5</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="3">
         <v>10</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="3">
         <v>18000</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="3">
         <v>22000</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="3">
         <v>5</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="3">
         <v>2</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K10" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="s">
+      <c r="A11" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="5">
         <v>25</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="5">
         <v>3500</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="5">
         <v>5000</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="5">
         <v>10</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="5">
         <v>3</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="s">
+      <c r="A12" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="3">
         <v>40</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="3">
         <v>3500</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="3">
         <v>5000</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="3">
         <v>15</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="3">
         <v>5</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="K12" t="s">
+      <c r="K12" s="2" t="s">
         <v>21</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="4"/>
+      <c r="K31" s="4"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="4"/>
+      <c r="K35" s="4"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5"/>
+      <c r="I39" s="5"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="4"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="4"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
+    </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" sqref="C2:C42" type="list">
+      <formula1>"sembako,minuman,snack,rokok,gas,kebutuhan,mie,bumbu,sayur,buah,obat,lainnya"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="D2:D42" type="list">
+      <formula1>"pcs,kg,liter,gram,bungkus,botol,karung,tabung,renceng,pax,lusin,rim"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(kios): normalize XLSX headers; update templates
</commit_message>
<xml_diff>
--- a/templates/produk-template.xlsx
+++ b/templates/produk-template.xlsx
@@ -8,172 +8,337 @@
   </bookViews>
   <sheets>
     <sheet name="Produk" sheetId="1" r:id="rId1"/>
+    <sheet name="Petunjuk" sheetId="2" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName hidden="true" localSheetId="0" name="_xlnm._FilterDatabase">'Produk'!$A$1:$K$42</definedName>
+  </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Kios Cerdas</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <t>⚠️ WAJIB DIISI
+Nama produk. Kunci pencocokan — nama sama = produk yang sama.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0">
+      <text>
+        <t>ℹ️ Opsional
+Kode barcode untuk scan/cari cepat. Boleh dikosongkan.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <t>ℹ️ Opsional
+Bebas (sembako, mie, minuman, dll). Pilih dari dropdown. Kosong → 'umum'.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <t>ℹ️ Opsional
+pcs/botol/karung/bungkus. Pilih dari dropdown. Kosong → 'pcs'.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
+      <text>
+        <t>ℹ️ Opsional
+Jumlah stok saat ini (angka positif).</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <t>ℹ️ Opsional
+Harga modal per satuan. Angka tanpa Rp/titik. Contoh: 55000</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <t>ℹ️ Opsional
+Harga jual per satuan. Angka tanpa Rp/titik.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
+      <text>
+        <t>ℹ️ Opsional
+Batas stok mulai diingatkan. Kosong → 5.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <t>ℹ️ Opsional
+Batas stok kritis/hampir habis. Kosong → 2.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0">
+      <text>
+        <t>ℹ️ Opsional
+Nama pemasok produk.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0">
+      <text>
+        <t>ℹ️ Opsional
+URL gambar produk (https://...) untuk tampil di toko pembeli. Boleh dikosongkan.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+  <si>
+    <t>nama *</t>
+  </si>
+  <si>
+    <t>barcode</t>
+  </si>
+  <si>
+    <t>kategori</t>
+  </si>
+  <si>
+    <t>satuan</t>
+  </si>
+  <si>
+    <t>stok</t>
+  </si>
+  <si>
+    <t>harga_beli</t>
+  </si>
+  <si>
+    <t>harga_jual</t>
+  </si>
+  <si>
+    <t>stok_minimum</t>
+  </si>
+  <si>
+    <t>stok_kritis</t>
+  </si>
+  <si>
+    <t>supplier</t>
+  </si>
+  <si>
+    <t>gambar</t>
+  </si>
+  <si>
+    <t>Beras Medium 5kg</t>
+  </si>
+  <si>
+    <t>8991234500015</t>
+  </si>
+  <si>
+    <t>sembako</t>
+  </si>
+  <si>
+    <t>karung</t>
+  </si>
+  <si>
+    <t>UD Maju</t>
+  </si>
+  <si>
+    <t>https://contoh.com/gambar/beras.jpg</t>
+  </si>
+  <si>
+    <t>Gula Pasir 1kg</t>
+  </si>
+  <si>
+    <t>8991234500022</t>
+  </si>
+  <si>
+    <t>bungkus</t>
+  </si>
+  <si>
+    <t>Distributor Kupang</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Minyak Goreng 1L</t>
+  </si>
+  <si>
+    <t>8991234500039</t>
+  </si>
+  <si>
+    <t>botol</t>
+  </si>
+  <si>
+    <t>Tepung Terigu 1kg</t>
+  </si>
+  <si>
+    <t>8991234500046</t>
+  </si>
+  <si>
+    <t>Indomie Goreng</t>
+  </si>
+  <si>
+    <t>089686010947</t>
+  </si>
+  <si>
+    <t>mie</t>
+  </si>
+  <si>
+    <t>pcs</t>
+  </si>
+  <si>
+    <t>Grosir Baa</t>
+  </si>
+  <si>
+    <t>Teh Botol 350ml</t>
+  </si>
+  <si>
+    <t>8992761111118</t>
+  </si>
+  <si>
+    <t>minuman</t>
+  </si>
+  <si>
+    <t>Kopi Sachet</t>
+  </si>
+  <si>
+    <t>renceng</t>
+  </si>
+  <si>
+    <t>Rokok Surya 16</t>
+  </si>
+  <si>
+    <t>8997011710018</t>
+  </si>
+  <si>
+    <t>rokok</t>
+  </si>
+  <si>
+    <t>Agen Rokok Rote</t>
+  </si>
+  <si>
+    <t>Gas LPG 3kg</t>
+  </si>
+  <si>
+    <t>gas</t>
+  </si>
+  <si>
+    <t>tabung</t>
+  </si>
+  <si>
+    <t>Pangkalan Gas Baa</t>
+  </si>
+  <si>
+    <t>Sabun Mandi</t>
+  </si>
+  <si>
+    <t>8999999036007</t>
+  </si>
+  <si>
+    <t>kebutuhan</t>
+  </si>
+  <si>
+    <t>Biskuit Kelapa</t>
+  </si>
+  <si>
+    <t>8990111222333</t>
+  </si>
+  <si>
+    <t>snack</t>
+  </si>
+  <si>
+    <t>Panduan Pengisian Template</t>
+  </si>
+  <si>
+    <t>Template ini untuk mengimport data produk ke Kios Cerdas.
+Isi kolom sesuai panduan, lalu simpan dan import via bot Telegram.</t>
+  </si>
+  <si>
+    <t>Kolom</t>
+  </si>
+  <si>
+    <t>Wajib?</t>
+  </si>
+  <si>
+    <t>Contoh</t>
+  </si>
+  <si>
+    <t>Keterangan</t>
+  </si>
+  <si>
+    <t>Validasi</t>
+  </si>
   <si>
     <t>nama</t>
   </si>
   <si>
-    <t>barcode</t>
-  </si>
-  <si>
-    <t>kategori</t>
-  </si>
-  <si>
-    <t>satuan</t>
-  </si>
-  <si>
-    <t>stok</t>
-  </si>
-  <si>
-    <t>harga_beli</t>
-  </si>
-  <si>
-    <t>harga_jual</t>
-  </si>
-  <si>
-    <t>stok_minimum</t>
-  </si>
-  <si>
-    <t>stok_kritis</t>
-  </si>
-  <si>
-    <t>supplier</t>
-  </si>
-  <si>
-    <t>gambar</t>
-  </si>
-  <si>
-    <t>Beras Medium 5kg</t>
-  </si>
-  <si>
-    <t>8991234500015</t>
-  </si>
-  <si>
-    <t>sembako</t>
-  </si>
-  <si>
-    <t>karung</t>
-  </si>
-  <si>
-    <t>UD Maju</t>
-  </si>
-  <si>
-    <t>https://contoh.com/gambar/beras.jpg</t>
-  </si>
-  <si>
-    <t>Gula Pasir 1kg</t>
-  </si>
-  <si>
-    <t>8991234500022</t>
-  </si>
-  <si>
-    <t>bungkus</t>
-  </si>
-  <si>
-    <t>Distributor Kupang</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Minyak Goreng 1L</t>
-  </si>
-  <si>
-    <t>8991234500039</t>
-  </si>
-  <si>
-    <t>botol</t>
-  </si>
-  <si>
-    <t>Tepung Terigu 1kg</t>
-  </si>
-  <si>
-    <t>8991234500046</t>
-  </si>
-  <si>
-    <t>Indomie Goreng</t>
-  </si>
-  <si>
-    <t>089686010947</t>
-  </si>
-  <si>
-    <t>mie</t>
-  </si>
-  <si>
-    <t>pcs</t>
-  </si>
-  <si>
-    <t>Grosir Baa</t>
-  </si>
-  <si>
-    <t>Teh Botol 350ml</t>
-  </si>
-  <si>
-    <t>8992761111118</t>
-  </si>
-  <si>
-    <t>minuman</t>
-  </si>
-  <si>
-    <t>Kopi Sachet</t>
-  </si>
-  <si>
-    <t>renceng</t>
-  </si>
-  <si>
-    <t>Rokok Surya 16</t>
-  </si>
-  <si>
-    <t>8997011710018</t>
-  </si>
-  <si>
-    <t>rokok</t>
-  </si>
-  <si>
-    <t>Agen Rokok Rote</t>
-  </si>
-  <si>
-    <t>Gas LPG 3kg</t>
-  </si>
-  <si>
-    <t>gas</t>
-  </si>
-  <si>
-    <t>tabung</t>
-  </si>
-  <si>
-    <t>Pangkalan Gas Baa</t>
-  </si>
-  <si>
-    <t>Sabun Mandi</t>
-  </si>
-  <si>
-    <t>8999999036007</t>
-  </si>
-  <si>
-    <t>kebutuhan</t>
-  </si>
-  <si>
-    <t>Biskuit Kelapa</t>
-  </si>
-  <si>
-    <t>8990111222333</t>
-  </si>
-  <si>
-    <t>snack</t>
+    <t>WAJIB</t>
+  </si>
+  <si>
+    <t>Nama produk. Kunci pencocokan — nama sama = produk yang sama.</t>
+  </si>
+  <si>
+    <t>Opsional</t>
+  </si>
+  <si>
+    <t>Kode barcode untuk scan/cari cepat. Boleh dikosongkan.</t>
+  </si>
+  <si>
+    <t>Bebas (sembako, mie, minuman, dll). Pilih dari dropdown. Kosong → 'umum'.</t>
+  </si>
+  <si>
+    <t>Pilih dari dropdown</t>
+  </si>
+  <si>
+    <t>pcs/botol/karung/bungkus. Pilih dari dropdown. Kosong → 'pcs'.</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Jumlah stok saat ini (angka positif).</t>
+  </si>
+  <si>
+    <t>Angka 0+ (tanpa Rp/titik)</t>
+  </si>
+  <si>
+    <t>55000</t>
+  </si>
+  <si>
+    <t>Harga modal per satuan. Angka tanpa Rp/titik. Contoh: 55000</t>
+  </si>
+  <si>
+    <t>62000</t>
+  </si>
+  <si>
+    <t>Harga jual per satuan. Angka tanpa Rp/titik.</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Batas stok mulai diingatkan. Kosong → 5.</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Batas stok kritis/hampir habis. Kosong → 2.</t>
+  </si>
+  <si>
+    <t>Nama pemasok produk.</t>
+  </si>
+  <si>
+    <t>URL gambar produk (https://...) untuk tampil di toko pembeli. Boleh dikosongkan.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -184,11 +349,34 @@
       <family val="2"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <family val="2"/>
+      <color rgb="FF2D3436"/>
       <sz val="11"/>
     </font>
     <font>
       <family val="2"/>
-      <color/>
+      <b val="1"/>
+      <color rgb="FF0D7C66"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <family val="2"/>
+      <color rgb="FF555555"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFC0392B"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -201,12 +389,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1B4F72"/>
+        <fgColor rgb="FF0D7C66"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD6EAF8"/>
+        <fgColor rgb="FFF0F7F4"/>
       </patternFill>
     </fill>
   </fills>
@@ -220,23 +408,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFBFC9CA"/>
+        <color rgb="FFCCDDC8"/>
       </left>
       <right style="thin">
-        <color rgb="FFBFC9CA"/>
+        <color rgb="FFCCDDC8"/>
       </right>
       <top style="thin">
-        <color rgb="FFBFC9CA"/>
+        <color rgb="FFCCDDC8"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFBFC9CA"/>
+        <color rgb="FFCCDDC8"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
@@ -252,6 +440,21 @@
     </xf>
     <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -520,6 +723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -531,10 +735,10 @@
     <col customWidth="true" max="7" min="6" width="16"/>
     <col customWidth="true" max="9" min="8" width="14"/>
     <col customWidth="true" max="10" min="10" width="22"/>
-    <col customWidth="true" max="11" min="11" width="42"/>
+    <col customWidth="true" max="11" min="11" width="38"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="true">
+    <row r="1" ht="32" customHeight="true">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1345,13 +1549,263 @@
       <c r="K42" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <autoFilter ref="$A$1:$K$42"/>
+  <dataValidations count="7">
     <dataValidation allowBlank="true" sqref="C2:C42" type="list">
       <formula1>"sembako,minuman,snack,rokok,gas,kebutuhan,mie,bumbu,sayur,buah,obat,lainnya"</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="D2:D42" type="list">
       <formula1>"pcs,kg,liter,gram,bungkus,botol,karung,tabung,renceng,pax,lusin,rim"</formula1>
     </dataValidation>
+    <dataValidation allowBlank="true" operator="greaterThanOrEqual" prompt="Masukkan angka 0 atau lebih. Tanpa Rp, tanpa titik. Contoh: 15000" promptTitle="Angka positif" showInputMessage="true" sqref="E2:E42" type="decimal">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" operator="greaterThanOrEqual" prompt="Masukkan angka 0 atau lebih. Tanpa Rp, tanpa titik. Contoh: 15000" promptTitle="Angka positif" showInputMessage="true" sqref="F2:F42" type="decimal">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" operator="greaterThanOrEqual" prompt="Masukkan angka 0 atau lebih. Tanpa Rp, tanpa titik. Contoh: 15000" promptTitle="Angka positif" showInputMessage="true" sqref="G2:G42" type="decimal">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" operator="greaterThanOrEqual" prompt="Masukkan angka 0 atau lebih. Tanpa Rp, tanpa titik. Contoh: 15000" promptTitle="Angka positif" showInputMessage="true" sqref="H2:H42" type="decimal">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" operator="greaterThanOrEqual" prompt="Masukkan angka 0 atau lebih. Tanpa Rp, tanpa titik. Contoh: 15000" promptTitle="Angka positif" showInputMessage="true" sqref="I2:I42" type="decimal">
+      <formula1>0</formula1>
+    </dataValidation>
   </dataValidations>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="22"/>
+    <col customWidth="true" max="2" min="2" width="12"/>
+    <col customWidth="true" max="3" min="3" width="40"/>
+    <col customWidth="true" max="4" min="4" width="46"/>
+    <col customWidth="true" max="5" min="5" width="24"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="true">
+      <c r="A1" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="true">
+      <c r="A2" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="true">
+      <c r="A5" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="true">
+      <c r="A6" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="true">
+      <c r="A7" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="true">
+      <c r="A8" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="true">
+      <c r="A9" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="true">
+      <c r="A10" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="true">
+      <c r="A11" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="true">
+      <c r="A12" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="true">
+      <c r="A13" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="true">
+      <c r="A14" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="true">
+      <c r="A15" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
 </worksheet>
 </file>
</xml_diff>